<commit_message>
chore: update code structure for better readability and maintainability
</commit_message>
<xml_diff>
--- a/Companies/Karat-CitiBank-Prep/Discussion_questions/Extras.xlsx
+++ b/Companies/Karat-CitiBank-Prep/Discussion_questions/Extras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work_USA\AIML\Projects\leetcode-solutions\Companies\Karat-CitiBank-Prep\Discussion_questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C89938C-7DD7-47BD-A590-76537ABCE3D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DA8DB1-9A03-4382-BD1E-EDD3CC6BA0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">Cpython? </t>
   </si>
@@ -686,6 +686,617 @@
       </rPr>
       <t>is the janitor that automatically cleans up objects once they are no longer referenced, ensuring the program doesn't run out of RAM.</t>
     </r>
+  </si>
+  <si>
+    <t>Whats @dataclass ?</t>
+  </si>
+  <si>
+    <t>To make a @dataclass immutable (read-only), you use the frozen=True parameter. This prevents fields from being modified after the object is created, which is excellent for data integrity in pipelines.
+from dataclasses import dataclass
+@dataclass(frozen=True)
+class User:
+    id: int
+    role: str
+u = User(1, "Admin")
+# u.role = "Editor"  &lt;-- This would raise a FrozenInstanceError</t>
+  </si>
+  <si>
+    <t>Iterator</t>
+  </si>
+  <si>
+    <t>An iterator is an object that allows you to traverse through a collection (like a list) one element at a time without loading everything into memory at once.</t>
+  </si>
+  <si>
+    <t>How would you design a machine learning model to detect fraudulent transactions in real-time for Citibank?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. The Core Problem: Imbalance &amp; Speed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Imbalance:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Fraud is rare (e.g., 99.9% of transactions are legit). If a model just guesses "Legit" every time, it gets 99.9% accuracy but catches 0% fraud. You must optimize for Recall (catching all fraud) over Accuracy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SLA (Service Level Agreement): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Credit card Swipes happen in milliseconds. The model must decide to "Approve" or "Deny" in under 100ms (often &lt;50ms) to avoid lagging the customer at the checkout.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">2. Feature Engineering (The Signal)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">To spot fraud instantly, you need "Contextual" features:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Velocity: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Is this the 5th transaction in 10 minutes?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Geo-distance: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Was the last swipe in New York and this one in London 20 minutes later? (Impossible travel).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Merchant Category:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Is a high-value electronics purchase unusual for this specific user profile</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5. The Real-time Stack</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+This is how data moves through Citibank's pipes:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">&gt; Kafka: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The "conveyor belt" that moves transaction data.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&gt; Redis (Feature Store):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> An ultra-fast in-memory database that stores the user's "last 5 minutes of activity" so the model can read it instantly.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">&gt; Triton/TorchServe: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Specialized servers that host the model and handle thousands of requests per second.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. The Two-Stage Architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+You don't run a heavy model on every single coffee purchase.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Stage 1 (Rules Engine): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Fast "If/Then" statements (e.g., "If amount &gt; $10k and new device, Block"). This handles the obvious cases in &lt;5ms.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Stage 2 (ML Model): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">For "grey area" cases, a fast model like XGBoost or LightGBM analyzes the patterns.
+Online Learning: Using River allows the model to learn from new fraud patterns as they happen in the stream, rather than waiting for a weekly retraining.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Handling Imbalance (The Math)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>F2 Score:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In fraud, a "False Negative" (missing a thief) is much more expensive than a "False Positive" (texting a customer to confirm a legit purchase). F2 weights Recall higher than Precision.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SMOTE/Class Weighting:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Techniques that tell the model, "Pay 100x more attention when you see a fraud example during training."</t>
+    </r>
+  </si>
+  <si>
+    <t>Describe optimizing a deep learning algorithm for performance and scalability.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. Training Efficiency (Saving GPU Memory &amp; Time)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Mixed Precision (FP16): Instead of using 32-bit numbers, use 16-bit. This cuts memory usage in half and speeds up math on modern GPUs (Tensor Cores).
+&gt; Gradient Checkpointing: Only save some "checkpoints" during the forward pass and re-calculate the rest during backpropagation. It saves RAM at the cost of a little extra computation.
+&gt; Gradient Accumulation: If your GPU is too small for a batch of 64, run 4 batches of 16 and only update the weights after the 4th run. It simulates a large batch on a small card.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Distributed Training (Scaling Across Multiple GPUs)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Data Parallelism (DDP): Every GPU has a full copy of the model, but they each look at different "shards" of data. They sync their gradients at the end.
+&gt; Model Parallelism: If the model is too big for one GPU (like GPT-4), you split the layers or tensors across multiple GPUs.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Inference Optimization (Speeding up Predictions)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Quantization (INT8): Converting weights from 32-bit floats to 8-bit integers. This drastically reduces model size and increases speed with minimal accuracy loss.
+&gt; ONNX + TensorRT: Exporting the model to a universal format (ONNX) and using NVIDIA’s TensorRT to "fuse" layers together, optimizing the math specifically for the GPU hardware.
+&gt; Model Distillation: Training a small "Student" model to mimic a massive "Teacher" model. You get a lightweight model that is much faster for production.
+&gt; KV-Cache: For Transformers (LLMs), this stores previous "keys and values" so the model doesn't re-calculate the entire sentence for every new word generated.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Scalability (Handling High Traffic)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Dynamic Batching (Triton): Instead of processing 1 request at a time, the server waits a few milliseconds to "group" incoming requests into a batch, which is much more efficient for the GPU.
+&gt; Kubernetes (K8s): Automatically spins up more "replicas" of your model server if traffic spikes and shuts them down when it's quiet to save money.</t>
+    </r>
+  </si>
+  <si>
+    <t>How would you design a photo-sharing app? Consider latency, throughput, and user scale.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. The Strategy: Decoupling &amp; CDNs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Edge Delivery: Use CloudFront (CDN) to cache photos globally. This ensures low latency regardless of where the user is located.
+&gt; Storage: Store original high-res photos in Amazon S3 (Blob Storage). Use Presigned URLs so the app can upload directly to S3, bypassing the main server to save bandwidth.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. The Write Path (Upload)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Asynchronous Processing: Uploads trigger a Kafka event. Background workers then handle the "heavy lifting" (generating thumbnails, resizing, and AI tagging) so the user doesn't have to wait.
+&gt; Metadata: Store the "who, when, and where" (file paths, tags) in PostgreSQL.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. The Read Path (Feed)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt; Caching: Use Redis to store the "Active User Feed." Retrieving a list of photo URLs from RAM is much faster than querying a database.
+&gt; Scalability: Use Cassandra for the activity timeline because it handles massive write volumes (likes, comments, follows) across multiple data centers.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Search &amp; Discovery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Elasticsearch: Sync metadata from Postgres to Elasticsearch to allow users to search for photos by tags or location instantly.</t>
+    </r>
+  </si>
+  <si>
+    <t>Design a comment system for a large website.</t>
   </si>
 </sst>
 </file>
@@ -709,12 +1320,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -729,12 +1346,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1017,7 +1637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B21"/>
+  <dimension ref="A2:B38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.36328125" style="2" customWidth="1"/>
@@ -1110,6 +1730,76 @@
         <v>20</v>
       </c>
     </row>
+    <row r="23" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="145" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="B28" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="87" x14ac:dyDescent="0.35">
+      <c r="B29" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="B32" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B33" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="116" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="87" x14ac:dyDescent="0.35">
+      <c r="B36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>